<commit_message>
[FIX] add various features to ris and stock replenishment
</commit_message>
<xml_diff>
--- a/dev/upmin_stock/static/template/procurement_data_import_template.xlsx
+++ b/dev/upmin_stock/static/template/procurement_data_import_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Japh\Documents\Work\UP Min QAO\odoo\odoo\dev\upmin_stock\static\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E82879DC-65BB-4761-A00B-00F211906328}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49CB76F6-0EAD-456B-AEFE-1CB0E2837571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -123,7 +123,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,6 +135,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -160,10 +168,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,7 +507,7 @@
       <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="2" t="s">
@@ -507,19 +516,19 @@
       <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="2" t="s">

</xml_diff>